<commit_message>
new cond file for new localizer design, one old localizer file for testing and new cond files for later learn and retrieval task
</commit_message>
<xml_diff>
--- a/psychopy_exp_files/sequences/block_conditions.xlsx
+++ b/psychopy_exp_files/sequences/block_conditions.xlsx
@@ -14,7 +14,7 @@
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913" iterateDelta="1E-4"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>condFileLearning</t>
   </si>
@@ -35,16 +35,28 @@
     <t>n_routes_block</t>
   </si>
   <si>
-    <t>sequences/learning_blockA_fixed-middle-10_0{participant_ID}.xlsx</t>
-  </si>
-  <si>
-    <t>sequences/learning_blockB_fixed-middle-10_0{participant_ID}.xlsx</t>
-  </si>
-  <si>
-    <t>sequences/retrieval_blockA_fixed-middle-10_0{participant_ID}.xlsx</t>
-  </si>
-  <si>
-    <t>sequences/retrieval_blockB_fixed-middle-10_0{participant_ID}.xlsx</t>
+    <t>sequences/learning_block1_fixed-middle-10_0{participant_ID}.xlsx</t>
+  </si>
+  <si>
+    <t>sequences/learning_block2_fixed-middle-10_0{participant_ID}.xlsx</t>
+  </si>
+  <si>
+    <t>sequences/learning_block3_fixed-middle-10_0{participant_ID}.xlsx</t>
+  </si>
+  <si>
+    <t>sequences/learning_block4_fixed-middle-10_0{participant_ID}.xlsx</t>
+  </si>
+  <si>
+    <t>sequences/retrieval_block1_fixed-middle-10_0{participant_ID}.xlsx</t>
+  </si>
+  <si>
+    <t>sequences/retrieval_block2_fixed-middle-10_0{participant_ID}.xlsx</t>
+  </si>
+  <si>
+    <t>sequences/retrieval_block3_fixed-middle-10_0{participant_ID}.xlsx</t>
+  </si>
+  <si>
+    <t>sequences/retrieval_block4_fixed-middle-10_0{participant_ID}.xlsx</t>
   </si>
 </sst>
 </file>
@@ -362,7 +374,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="32.33203125" customWidth="1"/>
@@ -385,10 +397,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C2">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -396,9 +408,31 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>6</v>
       </c>
-      <c r="C3">
+      <c r="B5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5">
         <v>4</v>
       </c>
     </row>

</xml_diff>